<commit_message>
data(listing-raw): ali 원본양식 갱신
</commit_message>
<xml_diff>
--- a/reference/listing_ali.xlsx
+++ b/reference/listing_ali.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr date1904="false"/>
-  <workbookProtection workbookAlgorithmName="MD5" workbookHashValue="q8pjal2ff5mRMWcJ4UtQeA==" workbookSaltValue="ZNm3TYHiWPRJ4XZdwOzpLw==" workbookSpinCount="100000" lockStructure="true"/>
+  <workbookProtection workbookAlgorithmName="MD5" workbookHashValue="/sVzCeafB0hPZETThJqePA==" workbookSaltValue="E7ki+FmZY9qvw5Psgg5S/A==" workbookSpinCount="100000" lockStructure="true"/>
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
@@ -27,18 +27,18 @@
     <sheet name="전통차건강음료_hide" r:id="rId20" sheetId="18" state="hidden"/>
     <sheet name="커피음료" r:id="rId21" sheetId="19"/>
     <sheet name="커피음료_hide" r:id="rId22" sheetId="20" state="hidden"/>
-    <sheet name="컵라면" r:id="rId23" sheetId="21"/>
-    <sheet name="컵라면_hide" r:id="rId24" sheetId="22" state="hidden"/>
-    <sheet name="올리브카퍼스" r:id="rId25" sheetId="23"/>
-    <sheet name="올리브카퍼스_hide" r:id="rId26" sheetId="24" state="hidden"/>
-    <sheet name="통조림옥수수" r:id="rId27" sheetId="25"/>
-    <sheet name="통조림옥수수_hide" r:id="rId28" sheetId="26" state="hidden"/>
-    <sheet name="미네랄워터" r:id="rId29" sheetId="27"/>
-    <sheet name="미네랄워터_hide" r:id="rId30" sheetId="28" state="hidden"/>
-    <sheet name="햄축산통조림" r:id="rId31" sheetId="29"/>
-    <sheet name="햄축산통조림_hide" r:id="rId32" sheetId="30" state="hidden"/>
-    <sheet name="통조림기타" r:id="rId33" sheetId="31"/>
-    <sheet name="통조림기타_hide" r:id="rId34" sheetId="32" state="hidden"/>
+    <sheet name="올리브카퍼스" r:id="rId23" sheetId="21"/>
+    <sheet name="올리브카퍼스_hide" r:id="rId24" sheetId="22" state="hidden"/>
+    <sheet name="통조림옥수수" r:id="rId25" sheetId="23"/>
+    <sheet name="통조림옥수수_hide" r:id="rId26" sheetId="24" state="hidden"/>
+    <sheet name="미네랄워터" r:id="rId27" sheetId="25"/>
+    <sheet name="미네랄워터_hide" r:id="rId28" sheetId="26" state="hidden"/>
+    <sheet name="햄축산통조림" r:id="rId29" sheetId="27"/>
+    <sheet name="햄축산통조림_hide" r:id="rId30" sheetId="28" state="hidden"/>
+    <sheet name="통조림기타" r:id="rId31" sheetId="29"/>
+    <sheet name="통조림기타_hide" r:id="rId32" sheetId="30" state="hidden"/>
+    <sheet name="컵라면" r:id="rId33" sheetId="31"/>
+    <sheet name="컵라면_hide" r:id="rId34" sheetId="32" state="hidden"/>
     <sheet name="통조림과일" r:id="rId35" sheetId="33"/>
     <sheet name="통조림과일_hide" r:id="rId36" sheetId="34" state="hidden"/>
     <sheet name="설탕대체" r:id="rId37" sheetId="35"/>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="F8" s="22" t="inlineStr">
         <is>
-          <t>9964</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="G8" s="22" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="F9" s="22" t="inlineStr">
         <is>
-          <t>9764</t>
+          <t>9759</t>
         </is>
       </c>
       <c r="G9" s="22" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t>9958</t>
+          <t>9957</t>
         </is>
       </c>
       <c r="G12" s="22" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="F13" s="22" t="inlineStr">
         <is>
-          <t>8613</t>
+          <t>8581</t>
         </is>
       </c>
       <c r="G13" s="22" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>9943</t>
+          <t>9942</t>
         </is>
       </c>
       <c r="G16" s="22" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="F19" s="22" t="inlineStr">
         <is>
-          <t>9996</t>
+          <t>9995</t>
         </is>
       </c>
       <c r="G19" s="22" t="inlineStr">
@@ -5478,12 +5478,12 @@
     <row r="31" customHeight="true" ht="30.0">
       <c r="A31" s="126" t="inlineStr">
         <is>
-          <t>1005007008459243</t>
+          <t>1005007043858234</t>
         </is>
       </c>
       <c r="B31" s="126" t="inlineStr">
         <is>
-          <t>CJ 스팸 클래식 1.81kg 6개</t>
+          <t>펭귄 백도 2절 400g 24개</t>
         </is>
       </c>
       <c r="C31" s="126" t="inlineStr">
@@ -5493,22 +5493,22 @@
       </c>
       <c r="D31" s="126" t="inlineStr">
         <is>
-          <t>12000039041916113</t>
+          <t>12000039203329259</t>
         </is>
       </c>
       <c r="E31" s="127" t="inlineStr">
         <is>
-          <t>145000.00</t>
+          <t>42300.00</t>
         </is>
       </c>
       <c r="F31" s="127" t="inlineStr">
         <is>
-          <t>932</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="G31" s="127" t="inlineStr">
         <is>
-          <t>15-05</t>
+          <t>14-04</t>
         </is>
       </c>
       <c r="H31" s="126"/>
@@ -5530,12 +5530,12 @@
     <row r="32" customHeight="true" ht="30.0">
       <c r="A32" s="126" t="inlineStr">
         <is>
-          <t>1005007043858234</t>
+          <t>1005007850567491</t>
         </is>
       </c>
       <c r="B32" s="126" t="inlineStr">
         <is>
-          <t>펭귄 백도 2절 400g 24개</t>
+          <t>펭귄 김치꽁치 380g 24개</t>
         </is>
       </c>
       <c r="C32" s="126" t="inlineStr">
@@ -5545,22 +5545,22 @@
       </c>
       <c r="D32" s="126" t="inlineStr">
         <is>
-          <t>12000039203329259</t>
+          <t>12000042534599714</t>
         </is>
       </c>
       <c r="E32" s="127" t="inlineStr">
         <is>
-          <t>42300.00</t>
+          <t>114200.00</t>
         </is>
       </c>
       <c r="F32" s="127" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G32" s="127" t="inlineStr">
         <is>
-          <t>14-04</t>
+          <t>11-05-02</t>
         </is>
       </c>
       <c r="H32" s="126"/>
@@ -5582,12 +5582,12 @@
     <row r="33" customHeight="true" ht="30.0">
       <c r="A33" s="126" t="inlineStr">
         <is>
-          <t>1005007850567491</t>
+          <t>1005007043625844</t>
         </is>
       </c>
       <c r="B33" s="126" t="inlineStr">
         <is>
-          <t>펭귄 김치꽁치 380g 24개</t>
+          <t>동원 자연산골뱅이 140g 48개</t>
         </is>
       </c>
       <c r="C33" s="126" t="inlineStr">
@@ -5597,12 +5597,12 @@
       </c>
       <c r="D33" s="126" t="inlineStr">
         <is>
-          <t>12000042534599714</t>
+          <t>12000039202863949</t>
         </is>
       </c>
       <c r="E33" s="127" t="inlineStr">
         <is>
-          <t>114200.00</t>
+          <t>153400.00</t>
         </is>
       </c>
       <c r="F33" s="127" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="G33" s="127" t="inlineStr">
         <is>
-          <t>11-05-02</t>
+          <t>11-16</t>
         </is>
       </c>
       <c r="H33" s="126"/>
@@ -5626,110 +5626,6 @@
       </c>
       <c r="M33" s="126"/>
       <c r="N33" s="126" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" customHeight="true" ht="30.0">
-      <c r="A34" s="126" t="inlineStr">
-        <is>
-          <t>1005007043625844</t>
-        </is>
-      </c>
-      <c r="B34" s="126" t="inlineStr">
-        <is>
-          <t>동원 자연산골뱅이 140g 48개</t>
-        </is>
-      </c>
-      <c r="C34" s="126" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D34" s="126" t="inlineStr">
-        <is>
-          <t>12000039202863949</t>
-        </is>
-      </c>
-      <c r="E34" s="127" t="inlineStr">
-        <is>
-          <t>153400.00</t>
-        </is>
-      </c>
-      <c r="F34" s="127" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G34" s="127" t="inlineStr">
-        <is>
-          <t>11-16</t>
-        </is>
-      </c>
-      <c r="H34" s="126"/>
-      <c r="I34" s="126"/>
-      <c r="J34" s="126"/>
-      <c r="K34" s="126"/>
-      <c r="L34" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M34" s="126"/>
-      <c r="N34" s="126" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" customHeight="true" ht="30.0">
-      <c r="A35" s="126" t="inlineStr">
-        <is>
-          <t>1005007044975012</t>
-        </is>
-      </c>
-      <c r="B35" s="126" t="inlineStr">
-        <is>
-          <t>한성 런천미트 200g 24개</t>
-        </is>
-      </c>
-      <c r="C35" s="126" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D35" s="126" t="inlineStr">
-        <is>
-          <t>12000039206135768</t>
-        </is>
-      </c>
-      <c r="E35" s="127" t="inlineStr">
-        <is>
-          <t>31900.00</t>
-        </is>
-      </c>
-      <c r="F35" s="127" t="inlineStr">
-        <is>
-          <t>9997</t>
-        </is>
-      </c>
-      <c r="G35" s="127" t="inlineStr">
-        <is>
-          <t>57-02</t>
-        </is>
-      </c>
-      <c r="H35" s="126"/>
-      <c r="I35" s="126"/>
-      <c r="J35" s="126"/>
-      <c r="K35" s="126"/>
-      <c r="L35" s="126" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M35" s="126"/>
-      <c r="N35" s="126" t="inlineStr">
         <is>
           <t>absolute</t>
         </is>
@@ -6672,7 +6568,7 @@
       </c>
       <c r="F6" s="148" t="inlineStr">
         <is>
-          <t>9966</t>
+          <t>9965</t>
         </is>
       </c>
       <c r="G6" s="148" t="inlineStr">
@@ -7837,7 +7733,7 @@
       </c>
       <c r="F6" s="169" t="inlineStr">
         <is>
-          <t>9886</t>
+          <t>9885</t>
         </is>
       </c>
       <c r="G6" s="169" t="inlineStr">
@@ -7941,7 +7837,7 @@
       </c>
       <c r="F8" s="169" t="inlineStr">
         <is>
-          <t>9448</t>
+          <t>9444</t>
         </is>
       </c>
       <c r="G8" s="169" t="inlineStr">
@@ -8409,7 +8305,7 @@
       </c>
       <c r="F17" s="169" t="inlineStr">
         <is>
-          <t>9857</t>
+          <t>9856</t>
         </is>
       </c>
       <c r="G17" s="169" t="inlineStr">
@@ -8769,7 +8665,7 @@
       </c>
       <c r="F23" s="169" t="inlineStr">
         <is>
-          <t>9946</t>
+          <t>9945</t>
         </is>
       </c>
       <c r="G23" s="169" t="inlineStr">
@@ -9237,7 +9133,7 @@
       </c>
       <c r="F32" s="169" t="inlineStr">
         <is>
-          <t>9924</t>
+          <t>9922</t>
         </is>
       </c>
       <c r="G32" s="169" t="inlineStr">
@@ -9445,7 +9341,7 @@
       </c>
       <c r="F36" s="169" t="inlineStr">
         <is>
-          <t>9795</t>
+          <t>9793</t>
         </is>
       </c>
       <c r="G36" s="169" t="inlineStr">
@@ -10173,7 +10069,7 @@
       </c>
       <c r="F50" s="169" t="inlineStr">
         <is>
-          <t>9928</t>
+          <t>9927</t>
         </is>
       </c>
       <c r="G50" s="169" t="inlineStr">
@@ -11362,7 +11258,7 @@
       </c>
       <c r="F6" s="190" t="inlineStr">
         <is>
-          <t>9849</t>
+          <t>9848</t>
         </is>
       </c>
       <c r="G6" s="190" t="inlineStr">
@@ -11466,7 +11362,7 @@
       </c>
       <c r="F8" s="190" t="inlineStr">
         <is>
-          <t>9814</t>
+          <t>9810</t>
         </is>
       </c>
       <c r="G8" s="190" t="inlineStr">
@@ -11570,7 +11466,7 @@
       </c>
       <c r="F10" s="190" t="inlineStr">
         <is>
-          <t>9859</t>
+          <t>9856</t>
         </is>
       </c>
       <c r="G10" s="190" t="inlineStr">
@@ -11778,7 +11674,7 @@
       </c>
       <c r="F14" s="190" t="inlineStr">
         <is>
-          <t>9826</t>
+          <t>9824</t>
         </is>
       </c>
       <c r="G14" s="190" t="inlineStr">
@@ -11882,7 +11778,7 @@
       </c>
       <c r="F16" s="190" t="inlineStr">
         <is>
-          <t>661</t>
+          <t>657</t>
         </is>
       </c>
       <c r="G16" s="190" t="inlineStr">
@@ -12174,7 +12070,7 @@
       </c>
       <c r="F21" s="190" t="inlineStr">
         <is>
-          <t>9924</t>
+          <t>9923</t>
         </is>
       </c>
       <c r="G21" s="190" t="inlineStr">
@@ -12382,7 +12278,7 @@
       </c>
       <c r="F25" s="190" t="inlineStr">
         <is>
-          <t>939</t>
+          <t>938</t>
         </is>
       </c>
       <c r="G25" s="190" t="inlineStr">
@@ -13006,7 +12902,7 @@
       </c>
       <c r="F37" s="190" t="inlineStr">
         <is>
-          <t>9979</t>
+          <t>9976</t>
         </is>
       </c>
       <c r="G37" s="190" t="inlineStr">
@@ -13162,7 +13058,7 @@
       </c>
       <c r="F40" s="190" t="inlineStr">
         <is>
-          <t>9860</t>
+          <t>9859</t>
         </is>
       </c>
       <c r="G40" s="190" t="inlineStr">
@@ -13214,7 +13110,7 @@
       </c>
       <c r="F41" s="190" t="inlineStr">
         <is>
-          <t>9976</t>
+          <t>9975</t>
         </is>
       </c>
       <c r="G41" s="190" t="inlineStr">
@@ -13578,7 +13474,7 @@
       </c>
       <c r="F48" s="190" t="inlineStr">
         <is>
-          <t>9869</t>
+          <t>9868</t>
         </is>
       </c>
       <c r="G48" s="190" t="inlineStr">
@@ -13838,7 +13734,7 @@
       </c>
       <c r="F53" s="190" t="inlineStr">
         <is>
-          <t>9962</t>
+          <t>9961</t>
         </is>
       </c>
       <c r="G53" s="190" t="inlineStr">
@@ -15339,7 +15235,7 @@
       </c>
       <c r="F6" s="211" t="inlineStr">
         <is>
-          <t>9937</t>
+          <t>9936</t>
         </is>
       </c>
       <c r="G6" s="211" t="inlineStr">
@@ -15391,7 +15287,7 @@
       </c>
       <c r="F7" s="211" t="inlineStr">
         <is>
-          <t>9974</t>
+          <t>9973</t>
         </is>
       </c>
       <c r="G7" s="211" t="inlineStr">
@@ -15807,7 +15703,7 @@
       </c>
       <c r="F15" s="211" t="inlineStr">
         <is>
-          <t>9909</t>
+          <t>9906</t>
         </is>
       </c>
       <c r="G15" s="211" t="inlineStr">
@@ -15859,7 +15755,7 @@
       </c>
       <c r="F16" s="211" t="inlineStr">
         <is>
-          <t>9748</t>
+          <t>9747</t>
         </is>
       </c>
       <c r="G16" s="211" t="inlineStr">
@@ -16015,7 +15911,7 @@
       </c>
       <c r="F19" s="211" t="inlineStr">
         <is>
-          <t>9971</t>
+          <t>9970</t>
         </is>
       </c>
       <c r="G19" s="211" t="inlineStr">
@@ -16067,7 +15963,7 @@
       </c>
       <c r="F20" s="211" t="inlineStr">
         <is>
-          <t>9973</t>
+          <t>9972</t>
         </is>
       </c>
       <c r="G20" s="211" t="inlineStr">
@@ -17861,12 +17757,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="231" t="inlineStr">
         <is>
-          <t>1005007044298727</t>
+          <t>1005007043774884</t>
         </is>
       </c>
       <c r="B6" s="231" t="inlineStr">
         <is>
-          <t>오뚜기 진라면 순한맛 멀티팩(5개입) 8개</t>
+          <t>동서 리치스 블랙 올리브 홀피티드3kg 5개</t>
         </is>
       </c>
       <c r="C6" s="231" t="inlineStr">
@@ -17876,44 +17772,28 @@
       </c>
       <c r="D6" s="231" t="inlineStr">
         <is>
-          <t>12000039205325343</t>
+          <t>12000039204139214</t>
         </is>
       </c>
       <c r="E6" s="232" t="inlineStr">
         <is>
-          <t>28100.00</t>
+          <t>99900.00</t>
         </is>
       </c>
       <c r="F6" s="232" t="inlineStr">
         <is>
-          <t>9843</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G6" s="232" t="inlineStr">
         <is>
-          <t>39-91-01</t>
-        </is>
-      </c>
-      <c r="H6" s="231" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I6" s="231" t="inlineStr">
-        <is>
-          <t>박스</t>
-        </is>
-      </c>
-      <c r="J6" s="231" t="inlineStr">
-        <is>
-          <t>4.80</t>
-        </is>
-      </c>
-      <c r="K6" s="231" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
+          <t>11-75-02</t>
+        </is>
+      </c>
+      <c r="H6" s="231"/>
+      <c r="I6" s="231"/>
+      <c r="J6" s="231"/>
+      <c r="K6" s="231"/>
       <c r="L6" s="231" t="inlineStr">
         <is>
           <t>-</t>
@@ -17921,318 +17801,6 @@
       </c>
       <c r="M6" s="231"/>
       <c r="N6" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" customHeight="true" ht="30.0">
-      <c r="A7" s="231" t="inlineStr">
-        <is>
-          <t>1005007044560498</t>
-        </is>
-      </c>
-      <c r="B7" s="231" t="inlineStr">
-        <is>
-          <t>농심 신라면 멀티팩(5개입) 8개</t>
-        </is>
-      </c>
-      <c r="C7" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D7" s="231" t="inlineStr">
-        <is>
-          <t>12000039205625151</t>
-        </is>
-      </c>
-      <c r="E7" s="232" t="inlineStr">
-        <is>
-          <t>35000.00</t>
-        </is>
-      </c>
-      <c r="F7" s="232" t="inlineStr">
-        <is>
-          <t>9951</t>
-        </is>
-      </c>
-      <c r="G7" s="232" t="inlineStr">
-        <is>
-          <t>54-01</t>
-        </is>
-      </c>
-      <c r="H7" s="231"/>
-      <c r="I7" s="231"/>
-      <c r="J7" s="231"/>
-      <c r="K7" s="231"/>
-      <c r="L7" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="231"/>
-      <c r="N7" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" customHeight="true" ht="30.0">
-      <c r="A8" s="231" t="inlineStr">
-        <is>
-          <t>1005007044473531</t>
-        </is>
-      </c>
-      <c r="B8" s="231" t="inlineStr">
-        <is>
-          <t>팔도 비빔면 멀티팩(5개입) 8개</t>
-        </is>
-      </c>
-      <c r="C8" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D8" s="231" t="inlineStr">
-        <is>
-          <t>12000039205412355</t>
-        </is>
-      </c>
-      <c r="E8" s="232" t="inlineStr">
-        <is>
-          <t>40000.00</t>
-        </is>
-      </c>
-      <c r="F8" s="232" t="inlineStr">
-        <is>
-          <t>9994</t>
-        </is>
-      </c>
-      <c r="G8" s="232" t="inlineStr">
-        <is>
-          <t>54-21</t>
-        </is>
-      </c>
-      <c r="H8" s="231"/>
-      <c r="I8" s="231"/>
-      <c r="J8" s="231"/>
-      <c r="K8" s="231"/>
-      <c r="L8" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="231"/>
-      <c r="N8" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customHeight="true" ht="30.0">
-      <c r="A9" s="231" t="inlineStr">
-        <is>
-          <t>1005007044527555</t>
-        </is>
-      </c>
-      <c r="B9" s="231" t="inlineStr">
-        <is>
-          <t>오뚜기 진라면 매운맛 멀티팩(5개입) 8개</t>
-        </is>
-      </c>
-      <c r="C9" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D9" s="231" t="inlineStr">
-        <is>
-          <t>12000039205101603</t>
-        </is>
-      </c>
-      <c r="E9" s="232" t="inlineStr">
-        <is>
-          <t>28100.00</t>
-        </is>
-      </c>
-      <c r="F9" s="232" t="inlineStr">
-        <is>
-          <t>9201</t>
-        </is>
-      </c>
-      <c r="G9" s="232" t="inlineStr">
-        <is>
-          <t>39-91</t>
-        </is>
-      </c>
-      <c r="H9" s="231"/>
-      <c r="I9" s="231"/>
-      <c r="J9" s="231"/>
-      <c r="K9" s="231"/>
-      <c r="L9" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="231"/>
-      <c r="N9" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" customHeight="true" ht="30.0">
-      <c r="A10" s="231" t="inlineStr">
-        <is>
-          <t>1005007044214904</t>
-        </is>
-      </c>
-      <c r="B10" s="231" t="inlineStr">
-        <is>
-          <t>팔도 왕뚜껑 컵라면 110g 18개</t>
-        </is>
-      </c>
-      <c r="C10" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D10" s="231" t="inlineStr">
-        <is>
-          <t>12000039205264392</t>
-        </is>
-      </c>
-      <c r="E10" s="232" t="inlineStr">
-        <is>
-          <t>23800.00</t>
-        </is>
-      </c>
-      <c r="F10" s="232" t="inlineStr">
-        <is>
-          <t>9966</t>
-        </is>
-      </c>
-      <c r="G10" s="232" t="inlineStr">
-        <is>
-          <t>22-22</t>
-        </is>
-      </c>
-      <c r="H10" s="231"/>
-      <c r="I10" s="231"/>
-      <c r="J10" s="231"/>
-      <c r="K10" s="231"/>
-      <c r="L10" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="231"/>
-      <c r="N10" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" customHeight="true" ht="30.0">
-      <c r="A11" s="231" t="inlineStr">
-        <is>
-          <t>1005007044375655</t>
-        </is>
-      </c>
-      <c r="B11" s="231" t="inlineStr">
-        <is>
-          <t>팔도 김치왕뚜껑 컵라면 18입</t>
-        </is>
-      </c>
-      <c r="C11" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D11" s="231" t="inlineStr">
-        <is>
-          <t>12000039205121918</t>
-        </is>
-      </c>
-      <c r="E11" s="232" t="inlineStr">
-        <is>
-          <t>23900.00</t>
-        </is>
-      </c>
-      <c r="F11" s="232" t="inlineStr">
-        <is>
-          <t>9994</t>
-        </is>
-      </c>
-      <c r="G11" s="232" t="inlineStr">
-        <is>
-          <t>22-23-01</t>
-        </is>
-      </c>
-      <c r="H11" s="231"/>
-      <c r="I11" s="231"/>
-      <c r="J11" s="231"/>
-      <c r="K11" s="231"/>
-      <c r="L11" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="231"/>
-      <c r="N11" s="231" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" customHeight="true" ht="30.0">
-      <c r="A12" s="231" t="inlineStr">
-        <is>
-          <t>1005007044267807</t>
-        </is>
-      </c>
-      <c r="B12" s="231" t="inlineStr">
-        <is>
-          <t>팔도 비빔면 컵라면 16입</t>
-        </is>
-      </c>
-      <c r="C12" s="231" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D12" s="231" t="inlineStr">
-        <is>
-          <t>12000039205464212</t>
-        </is>
-      </c>
-      <c r="E12" s="232" t="inlineStr">
-        <is>
-          <t>21500.00</t>
-        </is>
-      </c>
-      <c r="F12" s="232" t="inlineStr">
-        <is>
-          <t>9972</t>
-        </is>
-      </c>
-      <c r="G12" s="232" t="inlineStr">
-        <is>
-          <t>54-21-03</t>
-        </is>
-      </c>
-      <c r="H12" s="231"/>
-      <c r="I12" s="231"/>
-      <c r="J12" s="231"/>
-      <c r="K12" s="231"/>
-      <c r="L12" s="231" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M12" s="231"/>
-      <c r="N12" s="231" t="inlineStr">
         <is>
           <t>absolute</t>
         </is>
@@ -18243,10 +17811,10 @@
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(컵라면_hide!$I$7,0,0,5,1)</formula1>
+      <formula1>OFFSET(올리브카퍼스_hide!$I$7,0,0,5,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(컵라면_hide!$K$7,0,0,2,1)</formula1>
+      <formula1>OFFSET(올리브카퍼스_hide!$K$7,0,0,2,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -19110,12 +18678,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="252" t="inlineStr">
         <is>
-          <t>1005007043774884</t>
+          <t>1005007043714680</t>
         </is>
       </c>
       <c r="B6" s="252" t="inlineStr">
         <is>
-          <t>동서 리치스 블랙 올리브 홀피티드3kg 5개</t>
+          <t>동서 리치스홀커널스위트콘 소 (태국) 425g X 24캔</t>
         </is>
       </c>
       <c r="C6" s="252" t="inlineStr">
@@ -19125,22 +18693,22 @@
       </c>
       <c r="D6" s="252" t="inlineStr">
         <is>
-          <t>12000039204139214</t>
+          <t>12000039203736948</t>
         </is>
       </c>
       <c r="E6" s="253" t="inlineStr">
         <is>
-          <t>99900.00</t>
+          <t>26000.00</t>
         </is>
       </c>
       <c r="F6" s="253" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>9784</t>
         </is>
       </c>
       <c r="G6" s="253" t="inlineStr">
         <is>
-          <t>11-75-02</t>
+          <t>11-74-01</t>
         </is>
       </c>
       <c r="H6" s="252"/>
@@ -19159,15 +18727,119 @@
         </is>
       </c>
     </row>
+    <row r="7" customHeight="true" ht="30.0">
+      <c r="A7" s="252" t="inlineStr">
+        <is>
+          <t>1005007044083291</t>
+        </is>
+      </c>
+      <c r="B7" s="252" t="inlineStr">
+        <is>
+          <t>라리 스위트콘 덕용 2.95kg 5개</t>
+        </is>
+      </c>
+      <c r="C7" s="252" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" s="252" t="inlineStr">
+        <is>
+          <t>12000039203665747</t>
+        </is>
+      </c>
+      <c r="E7" s="253" t="inlineStr">
+        <is>
+          <t>42000.00</t>
+        </is>
+      </c>
+      <c r="F7" s="253" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="G7" s="253" t="inlineStr">
+        <is>
+          <t>11-73</t>
+        </is>
+      </c>
+      <c r="H7" s="252"/>
+      <c r="I7" s="252"/>
+      <c r="J7" s="252"/>
+      <c r="K7" s="252"/>
+      <c r="L7" s="252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="252"/>
+      <c r="N7" s="252" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" customHeight="true" ht="30.0">
+      <c r="A8" s="252" t="inlineStr">
+        <is>
+          <t>1005007008526120</t>
+        </is>
+      </c>
+      <c r="B8" s="252" t="inlineStr">
+        <is>
+          <t>동서 리치스 홀커널 스위트콘 덕용 (태국) 2,950kg 5개</t>
+        </is>
+      </c>
+      <c r="C8" s="252" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" s="252" t="inlineStr">
+        <is>
+          <t>12000039041685458</t>
+        </is>
+      </c>
+      <c r="E8" s="253" t="inlineStr">
+        <is>
+          <t>25100.00</t>
+        </is>
+      </c>
+      <c r="F8" s="253" t="inlineStr">
+        <is>
+          <t>9993</t>
+        </is>
+      </c>
+      <c r="G8" s="253" t="inlineStr">
+        <is>
+          <t>11-74</t>
+        </is>
+      </c>
+      <c r="H8" s="252"/>
+      <c r="I8" s="252"/>
+      <c r="J8" s="252"/>
+      <c r="K8" s="252"/>
+      <c r="L8" s="252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="252"/>
+      <c r="N8" s="252" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="true"/>
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(올리브카퍼스_hide!$I$7,0,0,5,1)</formula1>
+      <formula1>OFFSET(통조림옥수수_hide!$I$7,0,0,5,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(올리브카퍼스_hide!$K$7,0,0,2,1)</formula1>
+      <formula1>OFFSET(통조림옥수수_hide!$K$7,0,0,2,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -20031,12 +19703,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="273" t="inlineStr">
         <is>
-          <t>1005007043714680</t>
+          <t>1005007044397774</t>
         </is>
       </c>
       <c r="B6" s="273" t="inlineStr">
         <is>
-          <t>동서 리치스홀커널스위트콘 소 (태국) 425g X 24캔</t>
+          <t>동아제약 포카리스웨트 캔 245ml 30개</t>
         </is>
       </c>
       <c r="C6" s="273" t="inlineStr">
@@ -20046,22 +19718,22 @@
       </c>
       <c r="D6" s="273" t="inlineStr">
         <is>
-          <t>12000039203736948</t>
+          <t>12000039205577639</t>
         </is>
       </c>
       <c r="E6" s="274" t="inlineStr">
         <is>
-          <t>26000.00</t>
+          <t>23900.00</t>
         </is>
       </c>
       <c r="F6" s="274" t="inlineStr">
         <is>
-          <t>9786</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="G6" s="274" t="inlineStr">
         <is>
-          <t>11-74-01</t>
+          <t>28-01</t>
         </is>
       </c>
       <c r="H6" s="273"/>
@@ -20080,119 +19752,15 @@
         </is>
       </c>
     </row>
-    <row r="7" customHeight="true" ht="30.0">
-      <c r="A7" s="273" t="inlineStr">
-        <is>
-          <t>1005007044083291</t>
-        </is>
-      </c>
-      <c r="B7" s="273" t="inlineStr">
-        <is>
-          <t>라리 스위트콘 덕용 2.95kg 5개</t>
-        </is>
-      </c>
-      <c r="C7" s="273" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D7" s="273" t="inlineStr">
-        <is>
-          <t>12000039203665747</t>
-        </is>
-      </c>
-      <c r="E7" s="274" t="inlineStr">
-        <is>
-          <t>42000.00</t>
-        </is>
-      </c>
-      <c r="F7" s="274" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G7" s="274" t="inlineStr">
-        <is>
-          <t>11-73</t>
-        </is>
-      </c>
-      <c r="H7" s="273"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="273"/>
-      <c r="K7" s="273"/>
-      <c r="L7" s="273" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="273"/>
-      <c r="N7" s="273" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" customHeight="true" ht="30.0">
-      <c r="A8" s="273" t="inlineStr">
-        <is>
-          <t>1005007008526120</t>
-        </is>
-      </c>
-      <c r="B8" s="273" t="inlineStr">
-        <is>
-          <t>동서 리치스 홀커널 스위트콘 덕용 (태국) 2,950kg 5개</t>
-        </is>
-      </c>
-      <c r="C8" s="273" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D8" s="273" t="inlineStr">
-        <is>
-          <t>12000039041685458</t>
-        </is>
-      </c>
-      <c r="E8" s="274" t="inlineStr">
-        <is>
-          <t>25100.00</t>
-        </is>
-      </c>
-      <c r="F8" s="274" t="inlineStr">
-        <is>
-          <t>9993</t>
-        </is>
-      </c>
-      <c r="G8" s="274" t="inlineStr">
-        <is>
-          <t>11-74</t>
-        </is>
-      </c>
-      <c r="H8" s="273"/>
-      <c r="I8" s="273"/>
-      <c r="J8" s="273"/>
-      <c r="K8" s="273"/>
-      <c r="L8" s="273" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M8" s="273"/>
-      <c r="N8" s="273" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="true"/>
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(통조림옥수수_hide!$I$7,0,0,5,1)</formula1>
+      <formula1>OFFSET(미네랄워터_hide!$I$7,0,0,7,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(통조림옥수수_hide!$K$7,0,0,2,1)</formula1>
+      <formula1>OFFSET(미네랄워터_hide!$K$7,0,0,6,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -20407,13 +19975,13 @@
       <c r="H6"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J6"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="L6"/>
@@ -20431,7 +19999,7 @@
       <c r="H7"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>포장</t>
+          <t>병</t>
         </is>
       </c>
       <c r="J7"/>
@@ -20455,13 +20023,13 @@
       <c r="H8"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Piece（단품）</t>
+          <t>포장</t>
         </is>
       </c>
       <c r="J8"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>Fl oz</t>
         </is>
       </c>
       <c r="L8"/>
@@ -20479,13 +20047,13 @@
       <c r="H9"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>프로모션/기획 묶음</t>
+          <t>파우치 포장</t>
         </is>
       </c>
       <c r="J9"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>####splitter line####</t>
+          <t>L</t>
         </is>
       </c>
       <c r="L9"/>
@@ -20503,13 +20071,13 @@
       <c r="H10"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>박스</t>
+          <t>식품/병류 묶음 포장</t>
         </is>
       </c>
       <c r="J10"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>84498</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="L10"/>
@@ -20527,13 +20095,13 @@
       <c r="H11"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>세트</t>
+          <t>캔 포장 기준</t>
         </is>
       </c>
       <c r="J11"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>25237229774</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="L11"/>
@@ -20551,11 +20119,15 @@
       <c r="H12"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>####splitter line####</t>
+          <t>박스</t>
         </is>
       </c>
       <c r="J12"/>
-      <c r="K12"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
       <c r="L12"/>
       <c r="M12"/>
       <c r="N12"/>
@@ -20571,11 +20143,15 @@
       <c r="H13"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>6512378</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="J13"/>
-      <c r="K13"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>####splitter line####</t>
+        </is>
+      </c>
       <c r="L13"/>
       <c r="M13"/>
       <c r="N13"/>
@@ -20591,11 +20167,15 @@
       <c r="H14"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>7826584</t>
+          <t>####splitter line####</t>
         </is>
       </c>
       <c r="J14"/>
-      <c r="K14"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>84498</t>
+        </is>
+      </c>
       <c r="L14"/>
       <c r="M14"/>
       <c r="N14"/>
@@ -20611,11 +20191,15 @@
       <c r="H15"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>12301206</t>
+          <t>3525584</t>
         </is>
       </c>
       <c r="J15"/>
-      <c r="K15"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>1984039435</t>
+        </is>
+      </c>
       <c r="L15"/>
       <c r="M15"/>
       <c r="N15"/>
@@ -20631,11 +20215,15 @@
       <c r="H16"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23399605318</t>
+          <t>6512378</t>
         </is>
       </c>
       <c r="J16"/>
-      <c r="K16"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>21349054715</t>
+        </is>
+      </c>
       <c r="L16"/>
       <c r="M16"/>
       <c r="N16"/>
@@ -20651,14 +20239,106 @@
       <c r="H17"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>24087192969</t>
+          <t>8764850</t>
         </is>
       </c>
       <c r="J17"/>
-      <c r="K17"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>23313067566</t>
+        </is>
+      </c>
       <c r="L17"/>
       <c r="M17"/>
       <c r="N17"/>
+    </row>
+    <row r="18">
+      <c r="A18"/>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>37833420</t>
+        </is>
+      </c>
+      <c r="J18"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>23361021349</t>
+        </is>
+      </c>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+    </row>
+    <row r="19">
+      <c r="A19"/>
+      <c r="B19"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>22963608621</t>
+        </is>
+      </c>
+      <c r="J19"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>25237229774</t>
+        </is>
+      </c>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19"/>
+    </row>
+    <row r="20">
+      <c r="A20"/>
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>23399605318</t>
+        </is>
+      </c>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+    </row>
+    <row r="21">
+      <c r="A21"/>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="H21"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>24087192969</t>
+        </is>
+      </c>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -21056,12 +20736,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="294" t="inlineStr">
         <is>
-          <t>1005007044397774</t>
+          <t>1005007517558301</t>
         </is>
       </c>
       <c r="B6" s="294" t="inlineStr">
         <is>
-          <t>동아제약 포카리스웨트 캔 245ml 30개</t>
+          <t>스팸 8호 1세트 명절 추석 선물세트</t>
         </is>
       </c>
       <c r="C6" s="294" t="inlineStr">
@@ -21071,22 +20751,22 @@
       </c>
       <c r="D6" s="294" t="inlineStr">
         <is>
-          <t>12000039205577639</t>
+          <t>12000041099757732</t>
         </is>
       </c>
       <c r="E6" s="295" t="inlineStr">
         <is>
-          <t>23900.00</t>
+          <t>28900.00</t>
         </is>
       </c>
       <c r="F6" s="295" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>9953</t>
         </is>
       </c>
       <c r="G6" s="295" t="inlineStr">
         <is>
-          <t>28-01</t>
+          <t>45-21</t>
         </is>
       </c>
       <c r="H6" s="294"/>
@@ -21105,15 +20785,691 @@
         </is>
       </c>
     </row>
+    <row r="7" customHeight="true" ht="30.0">
+      <c r="A7" s="294" t="inlineStr">
+        <is>
+          <t>1005007517281893</t>
+        </is>
+      </c>
+      <c r="B7" s="294" t="inlineStr">
+        <is>
+          <t>스팸 8호 5세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C7" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D7" s="294" t="inlineStr">
+        <is>
+          <t>12000041099802360</t>
+        </is>
+      </c>
+      <c r="E7" s="295" t="inlineStr">
+        <is>
+          <t>130700.00</t>
+        </is>
+      </c>
+      <c r="F7" s="295" t="inlineStr">
+        <is>
+          <t>9760</t>
+        </is>
+      </c>
+      <c r="G7" s="295" t="inlineStr">
+        <is>
+          <t>45-21</t>
+        </is>
+      </c>
+      <c r="H7" s="294"/>
+      <c r="I7" s="294"/>
+      <c r="J7" s="294"/>
+      <c r="K7" s="294"/>
+      <c r="L7" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="294"/>
+      <c r="N7" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" customHeight="true" ht="30.0">
+      <c r="A8" s="294" t="inlineStr">
+        <is>
+          <t>1005007516909322</t>
+        </is>
+      </c>
+      <c r="B8" s="294" t="inlineStr">
+        <is>
+          <t>스팸복합2호 4세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C8" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D8" s="294" t="inlineStr">
+        <is>
+          <t>12000041098169615</t>
+        </is>
+      </c>
+      <c r="E8" s="295" t="inlineStr">
+        <is>
+          <t>113300.00</t>
+        </is>
+      </c>
+      <c r="F8" s="295" t="inlineStr">
+        <is>
+          <t>9904</t>
+        </is>
+      </c>
+      <c r="G8" s="295" t="inlineStr">
+        <is>
+          <t>45-27</t>
+        </is>
+      </c>
+      <c r="H8" s="294"/>
+      <c r="I8" s="294"/>
+      <c r="J8" s="294"/>
+      <c r="K8" s="294"/>
+      <c r="L8" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="294"/>
+      <c r="N8" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" customHeight="true" ht="30.0">
+      <c r="A9" s="294" t="inlineStr">
+        <is>
+          <t>1005007516965305</t>
+        </is>
+      </c>
+      <c r="B9" s="294" t="inlineStr">
+        <is>
+          <t>스팸복합2호 1세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C9" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D9" s="294" t="inlineStr">
+        <is>
+          <t>12000041097953976</t>
+        </is>
+      </c>
+      <c r="E9" s="295" t="inlineStr">
+        <is>
+          <t>30900.00</t>
+        </is>
+      </c>
+      <c r="F9" s="295" t="inlineStr">
+        <is>
+          <t>9988</t>
+        </is>
+      </c>
+      <c r="G9" s="295" t="inlineStr">
+        <is>
+          <t>45-27</t>
+        </is>
+      </c>
+      <c r="H9" s="294"/>
+      <c r="I9" s="294"/>
+      <c r="J9" s="294"/>
+      <c r="K9" s="294"/>
+      <c r="L9" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="294"/>
+      <c r="N9" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" customHeight="true" ht="30.0">
+      <c r="A10" s="294" t="inlineStr">
+        <is>
+          <t>1005010793399448</t>
+        </is>
+      </c>
+      <c r="B10" s="294" t="inlineStr">
+        <is>
+          <t>동원리챔g9호 1세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C10" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D10" s="294" t="inlineStr">
+        <is>
+          <t>12000053525229304</t>
+        </is>
+      </c>
+      <c r="E10" s="295" t="inlineStr">
+        <is>
+          <t>28600.00</t>
+        </is>
+      </c>
+      <c r="F10" s="295" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="G10" s="295" t="inlineStr">
+        <is>
+          <t>50-32</t>
+        </is>
+      </c>
+      <c r="H10" s="294"/>
+      <c r="I10" s="294"/>
+      <c r="J10" s="294"/>
+      <c r="K10" s="294"/>
+      <c r="L10" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="294"/>
+      <c r="N10" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" customHeight="true" ht="30.0">
+      <c r="A11" s="294" t="inlineStr">
+        <is>
+          <t>1005007517110036</t>
+        </is>
+      </c>
+      <c r="B11" s="294" t="inlineStr">
+        <is>
+          <t>스팸복합1호 5세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C11" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D11" s="294" t="inlineStr">
+        <is>
+          <t>12000041098274413</t>
+        </is>
+      </c>
+      <c r="E11" s="295" t="inlineStr">
+        <is>
+          <t>115000.00</t>
+        </is>
+      </c>
+      <c r="F11" s="295" t="inlineStr">
+        <is>
+          <t>9782</t>
+        </is>
+      </c>
+      <c r="G11" s="295" t="inlineStr">
+        <is>
+          <t>45-11</t>
+        </is>
+      </c>
+      <c r="H11" s="294"/>
+      <c r="I11" s="294"/>
+      <c r="J11" s="294"/>
+      <c r="K11" s="294"/>
+      <c r="L11" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" s="294"/>
+      <c r="N11" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" customHeight="true" ht="30.0">
+      <c r="A12" s="294" t="inlineStr">
+        <is>
+          <t>1005007517293809</t>
+        </is>
+      </c>
+      <c r="B12" s="294" t="inlineStr">
+        <is>
+          <t>동원리챔g9호 5세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C12" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D12" s="294" t="inlineStr">
+        <is>
+          <t>12000041099403698</t>
+        </is>
+      </c>
+      <c r="E12" s="295" t="inlineStr">
+        <is>
+          <t>129100.00</t>
+        </is>
+      </c>
+      <c r="F12" s="295" t="inlineStr">
+        <is>
+          <t>9987</t>
+        </is>
+      </c>
+      <c r="G12" s="295" t="inlineStr">
+        <is>
+          <t>50-32</t>
+        </is>
+      </c>
+      <c r="H12" s="294"/>
+      <c r="I12" s="294"/>
+      <c r="J12" s="294"/>
+      <c r="K12" s="294"/>
+      <c r="L12" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" s="294"/>
+      <c r="N12" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" customHeight="true" ht="30.0">
+      <c r="A13" s="294" t="inlineStr">
+        <is>
+          <t>1005007516996260</t>
+        </is>
+      </c>
+      <c r="B13" s="294" t="inlineStr">
+        <is>
+          <t>스팸복합1호 1세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C13" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D13" s="294" t="inlineStr">
+        <is>
+          <t>12000041098316444</t>
+        </is>
+      </c>
+      <c r="E13" s="295" t="inlineStr">
+        <is>
+          <t>25800.00</t>
+        </is>
+      </c>
+      <c r="F13" s="295" t="inlineStr">
+        <is>
+          <t>9989</t>
+        </is>
+      </c>
+      <c r="G13" s="295" t="inlineStr">
+        <is>
+          <t>45-11</t>
+        </is>
+      </c>
+      <c r="H13" s="294"/>
+      <c r="I13" s="294"/>
+      <c r="J13" s="294"/>
+      <c r="K13" s="294"/>
+      <c r="L13" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M13" s="294"/>
+      <c r="N13" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" customHeight="true" ht="30.0">
+      <c r="A14" s="294" t="inlineStr">
+        <is>
+          <t>1005007516954130</t>
+        </is>
+      </c>
+      <c r="B14" s="294" t="inlineStr">
+        <is>
+          <t>스팸3호 1세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C14" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D14" s="294" t="inlineStr">
+        <is>
+          <t>12000041097723983</t>
+        </is>
+      </c>
+      <c r="E14" s="295" t="inlineStr">
+        <is>
+          <t>51000.00</t>
+        </is>
+      </c>
+      <c r="F14" s="295" t="inlineStr">
+        <is>
+          <t>9991</t>
+        </is>
+      </c>
+      <c r="G14" s="295" t="inlineStr">
+        <is>
+          <t>45-10-01</t>
+        </is>
+      </c>
+      <c r="H14" s="294"/>
+      <c r="I14" s="294"/>
+      <c r="J14" s="294"/>
+      <c r="K14" s="294"/>
+      <c r="L14" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="294"/>
+      <c r="N14" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" customHeight="true" ht="30.0">
+      <c r="A15" s="294" t="inlineStr">
+        <is>
+          <t>1005011555929266</t>
+        </is>
+      </c>
+      <c r="B15" s="294" t="inlineStr">
+        <is>
+          <t>청정원 스페셜 S호 4세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C15" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D15" s="294" t="inlineStr">
+        <is>
+          <t>12000055911817125</t>
+        </is>
+      </c>
+      <c r="E15" s="295" t="inlineStr">
+        <is>
+          <t>54600.00</t>
+        </is>
+      </c>
+      <c r="F15" s="295" t="inlineStr">
+        <is>
+          <t>9961</t>
+        </is>
+      </c>
+      <c r="G15" s="295" t="inlineStr">
+        <is>
+          <t>01-19-10</t>
+        </is>
+      </c>
+      <c r="H15" s="294"/>
+      <c r="I15" s="294"/>
+      <c r="J15" s="294"/>
+      <c r="K15" s="294"/>
+      <c r="L15" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M15" s="294"/>
+      <c r="N15" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" customHeight="true" ht="30.0">
+      <c r="A16" s="294" t="inlineStr">
+        <is>
+          <t>1005011557386294</t>
+        </is>
+      </c>
+      <c r="B16" s="294" t="inlineStr">
+        <is>
+          <t>애경사랑 다온 14호 5세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C16" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D16" s="294" t="inlineStr">
+        <is>
+          <t>12000055914714451</t>
+        </is>
+      </c>
+      <c r="E16" s="295" t="inlineStr">
+        <is>
+          <t>58700.00</t>
+        </is>
+      </c>
+      <c r="F16" s="295" t="inlineStr">
+        <is>
+          <t>9960</t>
+        </is>
+      </c>
+      <c r="G16" s="295" t="inlineStr">
+        <is>
+          <t>45-20-+01</t>
+        </is>
+      </c>
+      <c r="H16" s="294"/>
+      <c r="I16" s="294"/>
+      <c r="J16" s="294"/>
+      <c r="K16" s="294"/>
+      <c r="L16" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M16" s="294"/>
+      <c r="N16" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" customHeight="true" ht="30.0">
+      <c r="A17" s="294" t="inlineStr">
+        <is>
+          <t>1005010793311780</t>
+        </is>
+      </c>
+      <c r="B17" s="294" t="inlineStr">
+        <is>
+          <t>동원 스페셜 5호 1세트 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C17" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D17" s="294" t="inlineStr">
+        <is>
+          <t>12000053525115949</t>
+        </is>
+      </c>
+      <c r="E17" s="295" t="inlineStr">
+        <is>
+          <t>24600.00</t>
+        </is>
+      </c>
+      <c r="F17" s="295" t="inlineStr">
+        <is>
+          <t>9981</t>
+        </is>
+      </c>
+      <c r="G17" s="295" t="inlineStr">
+        <is>
+          <t>50-71-02</t>
+        </is>
+      </c>
+      <c r="H17" s="294"/>
+      <c r="I17" s="294"/>
+      <c r="J17" s="294"/>
+      <c r="K17" s="294"/>
+      <c r="L17" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" s="294"/>
+      <c r="N17" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" customHeight="true" ht="30.0">
+      <c r="A18" s="294" t="inlineStr">
+        <is>
+          <t>1005007517486374</t>
+        </is>
+      </c>
+      <c r="B18" s="294" t="inlineStr">
+        <is>
+          <t>스팸6호 4세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C18" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D18" s="294" t="inlineStr">
+        <is>
+          <t>12000041099568766</t>
+        </is>
+      </c>
+      <c r="E18" s="295" t="inlineStr">
+        <is>
+          <t>154500.00</t>
+        </is>
+      </c>
+      <c r="F18" s="295" t="inlineStr">
+        <is>
+          <t>9816</t>
+        </is>
+      </c>
+      <c r="G18" s="295" t="inlineStr">
+        <is>
+          <t>45-05</t>
+        </is>
+      </c>
+      <c r="H18" s="294"/>
+      <c r="I18" s="294"/>
+      <c r="J18" s="294"/>
+      <c r="K18" s="294"/>
+      <c r="L18" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" s="294"/>
+      <c r="N18" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" customHeight="true" ht="30.0">
+      <c r="A19" s="294" t="inlineStr">
+        <is>
+          <t>1005007517580171</t>
+        </is>
+      </c>
+      <c r="B19" s="294" t="inlineStr">
+        <is>
+          <t>스팸6호 1세트 스팸 명절 추석 선물세트</t>
+        </is>
+      </c>
+      <c r="C19" s="294" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="D19" s="294" t="inlineStr">
+        <is>
+          <t>12000041099919070</t>
+        </is>
+      </c>
+      <c r="E19" s="295" t="inlineStr">
+        <is>
+          <t>41200.00</t>
+        </is>
+      </c>
+      <c r="F19" s="295" t="inlineStr">
+        <is>
+          <t>9916</t>
+        </is>
+      </c>
+      <c r="G19" s="295" t="inlineStr">
+        <is>
+          <t>45-05</t>
+        </is>
+      </c>
+      <c r="H19" s="294"/>
+      <c r="I19" s="294"/>
+      <c r="J19" s="294"/>
+      <c r="K19" s="294"/>
+      <c r="L19" s="294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" s="294"/>
+      <c r="N19" s="294" t="inlineStr">
+        <is>
+          <t>absolute</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="true"/>
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(미네랄워터_hide!$I$7,0,0,7,1)</formula1>
+      <formula1>OFFSET(햄축산통조림_hide!$I$7,0,0,6,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(미네랄워터_hide!$K$7,0,0,6,1)</formula1>
+      <formula1>OFFSET(햄축산통조림_hide!$K$7,0,0,2,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -21328,13 +21684,13 @@
       <c r="H6"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J6"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L6"/>
@@ -21382,7 +21738,7 @@
       <c r="J8"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Fl oz</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="L8"/>
@@ -21400,13 +21756,13 @@
       <c r="H9"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>파우치 포장</t>
+          <t>Piece（단품）</t>
         </is>
       </c>
       <c r="J9"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>####splitter line####</t>
         </is>
       </c>
       <c r="L9"/>
@@ -21424,13 +21780,13 @@
       <c r="H10"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>식품/병류 묶음 포장</t>
+          <t>프로모션/기획 묶음</t>
         </is>
       </c>
       <c r="J10"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>84498</t>
         </is>
       </c>
       <c r="L10"/>
@@ -21448,13 +21804,13 @@
       <c r="H11"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>캔 포장 기준</t>
+          <t>박스</t>
         </is>
       </c>
       <c r="J11"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>25237229774</t>
         </is>
       </c>
       <c r="L11"/>
@@ -21472,15 +21828,11 @@
       <c r="H12"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>박스</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="J12"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
+      <c r="K12"/>
       <c r="L12"/>
       <c r="M12"/>
       <c r="N12"/>
@@ -21496,15 +21848,11 @@
       <c r="H13"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>세트</t>
+          <t>####splitter line####</t>
         </is>
       </c>
       <c r="J13"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>####splitter line####</t>
-        </is>
-      </c>
+      <c r="K13"/>
       <c r="L13"/>
       <c r="M13"/>
       <c r="N13"/>
@@ -21520,15 +21868,11 @@
       <c r="H14"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>####splitter line####</t>
+          <t>3525584</t>
         </is>
       </c>
       <c r="J14"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>84498</t>
-        </is>
-      </c>
+      <c r="K14"/>
       <c r="L14"/>
       <c r="M14"/>
       <c r="N14"/>
@@ -21544,15 +21888,11 @@
       <c r="H15"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3525584</t>
+          <t>6512378</t>
         </is>
       </c>
       <c r="J15"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>1984039435</t>
-        </is>
-      </c>
+      <c r="K15"/>
       <c r="L15"/>
       <c r="M15"/>
       <c r="N15"/>
@@ -21568,15 +21908,11 @@
       <c r="H16"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>6512378</t>
+          <t>7826584</t>
         </is>
       </c>
       <c r="J16"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>21349054715</t>
-        </is>
-      </c>
+      <c r="K16"/>
       <c r="L16"/>
       <c r="M16"/>
       <c r="N16"/>
@@ -21592,15 +21928,11 @@
       <c r="H17"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>8764850</t>
+          <t>12301206</t>
         </is>
       </c>
       <c r="J17"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>23313067566</t>
-        </is>
-      </c>
+      <c r="K17"/>
       <c r="L17"/>
       <c r="M17"/>
       <c r="N17"/>
@@ -21616,15 +21948,11 @@
       <c r="H18"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>37833420</t>
+          <t>23399605318</t>
         </is>
       </c>
       <c r="J18"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>23361021349</t>
-        </is>
-      </c>
+      <c r="K18"/>
       <c r="L18"/>
       <c r="M18"/>
       <c r="N18"/>
@@ -21640,58 +21968,14 @@
       <c r="H19"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>22963608621</t>
+          <t>24087192969</t>
         </is>
       </c>
       <c r="J19"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>25237229774</t>
-        </is>
-      </c>
+      <c r="K19"/>
       <c r="L19"/>
       <c r="M19"/>
       <c r="N19"/>
-    </row>
-    <row r="20">
-      <c r="A20"/>
-      <c r="B20"/>
-      <c r="C20"/>
-      <c r="D20"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>23399605318</t>
-        </is>
-      </c>
-      <c r="J20"/>
-      <c r="K20"/>
-      <c r="L20"/>
-      <c r="M20"/>
-      <c r="N20"/>
-    </row>
-    <row r="21">
-      <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>24087192969</t>
-        </is>
-      </c>
-      <c r="J21"/>
-      <c r="K21"/>
-      <c r="L21"/>
-      <c r="M21"/>
-      <c r="N21"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -22089,12 +22373,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="315" t="inlineStr">
         <is>
-          <t>1005007517558301</t>
+          <t>1005009937710715</t>
         </is>
       </c>
       <c r="B6" s="315" t="inlineStr">
         <is>
-          <t>스팸 8호 1세트 명절 추석 선물세트</t>
+          <t>스팸 특별한선택 H-2호 5세트 선물세트</t>
         </is>
       </c>
       <c r="C6" s="315" t="inlineStr">
@@ -22104,22 +22388,22 @@
       </c>
       <c r="D6" s="315" t="inlineStr">
         <is>
-          <t>12000041099757732</t>
+          <t>12000050627105859</t>
         </is>
       </c>
       <c r="E6" s="316" t="inlineStr">
         <is>
-          <t>28900.00</t>
+          <t>79900.00</t>
         </is>
       </c>
       <c r="F6" s="316" t="inlineStr">
         <is>
-          <t>9954</t>
+          <t>9996</t>
         </is>
       </c>
       <c r="G6" s="316" t="inlineStr">
         <is>
-          <t>45-21</t>
+          <t>45-12-06</t>
         </is>
       </c>
       <c r="H6" s="315"/>
@@ -22141,12 +22425,12 @@
     <row r="7" customHeight="true" ht="30.0">
       <c r="A7" s="315" t="inlineStr">
         <is>
-          <t>1005007517281893</t>
+          <t>1005009943428343</t>
         </is>
       </c>
       <c r="B7" s="315" t="inlineStr">
         <is>
-          <t>스팸 8호 5세트 명절 추석 선물세트</t>
+          <t>스팸 특별한선택 H-2호 1세트 선물세트</t>
         </is>
       </c>
       <c r="C7" s="315" t="inlineStr">
@@ -22156,22 +22440,22 @@
       </c>
       <c r="D7" s="315" t="inlineStr">
         <is>
-          <t>12000041099802360</t>
+          <t>12000050643623167</t>
         </is>
       </c>
       <c r="E7" s="316" t="inlineStr">
         <is>
-          <t>130700.00</t>
+          <t>18700.00</t>
         </is>
       </c>
       <c r="F7" s="316" t="inlineStr">
         <is>
-          <t>9760</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G7" s="316" t="inlineStr">
         <is>
-          <t>45-21</t>
+          <t>45-12-06</t>
         </is>
       </c>
       <c r="H7" s="315"/>
@@ -22193,12 +22477,12 @@
     <row r="8" customHeight="true" ht="30.0">
       <c r="A8" s="315" t="inlineStr">
         <is>
-          <t>1005007516909322</t>
+          <t>1005009943395385</t>
         </is>
       </c>
       <c r="B8" s="315" t="inlineStr">
         <is>
-          <t>스팸복합2호 4세트 스팸 명절 추석 선물세트</t>
+          <t>스팸 12K호 1세트</t>
         </is>
       </c>
       <c r="C8" s="315" t="inlineStr">
@@ -22208,22 +22492,22 @@
       </c>
       <c r="D8" s="315" t="inlineStr">
         <is>
-          <t>12000041098169615</t>
+          <t>12000050643682021</t>
         </is>
       </c>
       <c r="E8" s="316" t="inlineStr">
         <is>
-          <t>113300.00</t>
+          <t>26500.00</t>
         </is>
       </c>
       <c r="F8" s="316" t="inlineStr">
         <is>
-          <t>9904</t>
+          <t>9997</t>
         </is>
       </c>
       <c r="G8" s="316" t="inlineStr">
         <is>
-          <t>45-27</t>
+          <t>45-10-09</t>
         </is>
       </c>
       <c r="H8" s="315"/>
@@ -22245,12 +22529,12 @@
     <row r="9" customHeight="true" ht="30.0">
       <c r="A9" s="315" t="inlineStr">
         <is>
-          <t>1005007516965305</t>
+          <t>1005009937638801</t>
         </is>
       </c>
       <c r="B9" s="315" t="inlineStr">
         <is>
-          <t>스팸복합2호 1세트 스팸 명절 추석 선물세트</t>
+          <t>스팸 12K호 4세트</t>
         </is>
       </c>
       <c r="C9" s="315" t="inlineStr">
@@ -22260,22 +22544,22 @@
       </c>
       <c r="D9" s="315" t="inlineStr">
         <is>
-          <t>12000041097953976</t>
+          <t>12000050627038470</t>
         </is>
       </c>
       <c r="E9" s="316" t="inlineStr">
         <is>
-          <t>30900.00</t>
+          <t>95500.00</t>
         </is>
       </c>
       <c r="F9" s="316" t="inlineStr">
         <is>
-          <t>9988</t>
+          <t>9942</t>
         </is>
       </c>
       <c r="G9" s="316" t="inlineStr">
         <is>
-          <t>45-27</t>
+          <t>45-10-09</t>
         </is>
       </c>
       <c r="H9" s="315"/>
@@ -22297,12 +22581,12 @@
     <row r="10" customHeight="true" ht="30.0">
       <c r="A10" s="315" t="inlineStr">
         <is>
-          <t>1005010793399448</t>
+          <t>1005009937881801</t>
         </is>
       </c>
       <c r="B10" s="315" t="inlineStr">
         <is>
-          <t>동원리챔g9호 1세트 명절 추석 선물세트</t>
+          <t>CJ 풍성한S호 3세트 선물세트</t>
         </is>
       </c>
       <c r="C10" s="315" t="inlineStr">
@@ -22312,12 +22596,12 @@
       </c>
       <c r="D10" s="315" t="inlineStr">
         <is>
-          <t>12000053525229304</t>
+          <t>12000050627580842</t>
         </is>
       </c>
       <c r="E10" s="316" t="inlineStr">
         <is>
-          <t>28600.00</t>
+          <t>133300.00</t>
         </is>
       </c>
       <c r="F10" s="316" t="inlineStr">
@@ -22327,7 +22611,7 @@
       </c>
       <c r="G10" s="316" t="inlineStr">
         <is>
-          <t>50-32</t>
+          <t>45-09-01</t>
         </is>
       </c>
       <c r="H10" s="315"/>
@@ -22349,12 +22633,12 @@
     <row r="11" customHeight="true" ht="30.0">
       <c r="A11" s="315" t="inlineStr">
         <is>
-          <t>1005007517110036</t>
+          <t>1005009943444204</t>
         </is>
       </c>
       <c r="B11" s="315" t="inlineStr">
         <is>
-          <t>스팸복합1호 5세트 스팸 명절 추석 선물세트</t>
+          <t>청정원 스페셜 NH2호 1세트 선물세트</t>
         </is>
       </c>
       <c r="C11" s="315" t="inlineStr">
@@ -22364,22 +22648,22 @@
       </c>
       <c r="D11" s="315" t="inlineStr">
         <is>
-          <t>12000041098274413</t>
+          <t>12000050643525722</t>
         </is>
       </c>
       <c r="E11" s="316" t="inlineStr">
         <is>
-          <t>115000.00</t>
+          <t>27500.00</t>
         </is>
       </c>
       <c r="F11" s="316" t="inlineStr">
         <is>
-          <t>9782</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G11" s="316" t="inlineStr">
         <is>
-          <t>45-11</t>
+          <t>01-17</t>
         </is>
       </c>
       <c r="H11" s="315"/>
@@ -22401,12 +22685,12 @@
     <row r="12" customHeight="true" ht="30.0">
       <c r="A12" s="315" t="inlineStr">
         <is>
-          <t>1005007517293809</t>
+          <t>1005009937891554</t>
         </is>
       </c>
       <c r="B12" s="315" t="inlineStr">
         <is>
-          <t>동원리챔g9호 5세트 명절 추석 선물세트</t>
+          <t>청정원 스페셜 NH2호 3세트 선물세트</t>
         </is>
       </c>
       <c r="C12" s="315" t="inlineStr">
@@ -22416,22 +22700,22 @@
       </c>
       <c r="D12" s="315" t="inlineStr">
         <is>
-          <t>12000041099403698</t>
+          <t>12000050627562432</t>
         </is>
       </c>
       <c r="E12" s="316" t="inlineStr">
         <is>
-          <t>129100.00</t>
+          <t>75700.00</t>
         </is>
       </c>
       <c r="F12" s="316" t="inlineStr">
         <is>
-          <t>9987</t>
+          <t>9995</t>
         </is>
       </c>
       <c r="G12" s="316" t="inlineStr">
         <is>
-          <t>50-32</t>
+          <t>01-17</t>
         </is>
       </c>
       <c r="H12" s="315"/>
@@ -22453,12 +22737,12 @@
     <row r="13" customHeight="true" ht="30.0">
       <c r="A13" s="315" t="inlineStr">
         <is>
-          <t>1005007516996260</t>
+          <t>1005009943250846</t>
         </is>
       </c>
       <c r="B13" s="315" t="inlineStr">
         <is>
-          <t>스팸복합1호 1세트 스팸 명절 추석 선물세트</t>
+          <t>청정원 L6호 1세트 선물세트</t>
         </is>
       </c>
       <c r="C13" s="315" t="inlineStr">
@@ -22468,22 +22752,22 @@
       </c>
       <c r="D13" s="315" t="inlineStr">
         <is>
-          <t>12000041098316444</t>
+          <t>12000050643481691</t>
         </is>
       </c>
       <c r="E13" s="316" t="inlineStr">
         <is>
-          <t>25800.00</t>
+          <t>23200.00</t>
         </is>
       </c>
       <c r="F13" s="316" t="inlineStr">
         <is>
-          <t>9989</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G13" s="316" t="inlineStr">
         <is>
-          <t>45-11</t>
+          <t>01-19-06</t>
         </is>
       </c>
       <c r="H13" s="315"/>
@@ -22505,12 +22789,12 @@
     <row r="14" customHeight="true" ht="30.0">
       <c r="A14" s="315" t="inlineStr">
         <is>
-          <t>1005007516954130</t>
+          <t>1005009937925088</t>
         </is>
       </c>
       <c r="B14" s="315" t="inlineStr">
         <is>
-          <t>스팸3호 1세트 스팸 명절 추석 선물세트</t>
+          <t>청정원 L6호 4세트 선물세트</t>
         </is>
       </c>
       <c r="C14" s="315" t="inlineStr">
@@ -22520,22 +22804,22 @@
       </c>
       <c r="D14" s="315" t="inlineStr">
         <is>
-          <t>12000041097723983</t>
+          <t>12000050627510269</t>
         </is>
       </c>
       <c r="E14" s="316" t="inlineStr">
         <is>
-          <t>51000.00</t>
+          <t>82700.00</t>
         </is>
       </c>
       <c r="F14" s="316" t="inlineStr">
         <is>
-          <t>9991</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G14" s="316" t="inlineStr">
         <is>
-          <t>45-10-01</t>
+          <t>01-19-06</t>
         </is>
       </c>
       <c r="H14" s="315"/>
@@ -22557,12 +22841,12 @@
     <row r="15" customHeight="true" ht="30.0">
       <c r="A15" s="315" t="inlineStr">
         <is>
-          <t>1005011555929266</t>
+          <t>1005007850275922</t>
         </is>
       </c>
       <c r="B15" s="315" t="inlineStr">
         <is>
-          <t>청정원 스페셜 S호 4세트 명절 추석 선물세트</t>
+          <t>동표 을지로골뱅이 400g 24개</t>
         </is>
       </c>
       <c r="C15" s="315" t="inlineStr">
@@ -22572,22 +22856,22 @@
       </c>
       <c r="D15" s="315" t="inlineStr">
         <is>
-          <t>12000055911817125</t>
+          <t>12000042534092495</t>
         </is>
       </c>
       <c r="E15" s="316" t="inlineStr">
         <is>
-          <t>54600.00</t>
+          <t>189300.00</t>
         </is>
       </c>
       <c r="F15" s="316" t="inlineStr">
         <is>
-          <t>9961</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="G15" s="316" t="inlineStr">
         <is>
-          <t>01-19-10</t>
+          <t>46-04</t>
         </is>
       </c>
       <c r="H15" s="315"/>
@@ -22606,223 +22890,15 @@
         </is>
       </c>
     </row>
-    <row r="16" customHeight="true" ht="30.0">
-      <c r="A16" s="315" t="inlineStr">
-        <is>
-          <t>1005011557386294</t>
-        </is>
-      </c>
-      <c r="B16" s="315" t="inlineStr">
-        <is>
-          <t>애경사랑 다온 14호 5세트 명절 추석 선물세트</t>
-        </is>
-      </c>
-      <c r="C16" s="315" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D16" s="315" t="inlineStr">
-        <is>
-          <t>12000055914714451</t>
-        </is>
-      </c>
-      <c r="E16" s="316" t="inlineStr">
-        <is>
-          <t>58700.00</t>
-        </is>
-      </c>
-      <c r="F16" s="316" t="inlineStr">
-        <is>
-          <t>9960</t>
-        </is>
-      </c>
-      <c r="G16" s="316" t="inlineStr">
-        <is>
-          <t>45-20-+01</t>
-        </is>
-      </c>
-      <c r="H16" s="315"/>
-      <c r="I16" s="315"/>
-      <c r="J16" s="315"/>
-      <c r="K16" s="315"/>
-      <c r="L16" s="315" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M16" s="315"/>
-      <c r="N16" s="315" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" customHeight="true" ht="30.0">
-      <c r="A17" s="315" t="inlineStr">
-        <is>
-          <t>1005010793311780</t>
-        </is>
-      </c>
-      <c r="B17" s="315" t="inlineStr">
-        <is>
-          <t>동원 스페셜 5호 1세트 명절 추석 선물세트</t>
-        </is>
-      </c>
-      <c r="C17" s="315" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D17" s="315" t="inlineStr">
-        <is>
-          <t>12000053525115949</t>
-        </is>
-      </c>
-      <c r="E17" s="316" t="inlineStr">
-        <is>
-          <t>24600.00</t>
-        </is>
-      </c>
-      <c r="F17" s="316" t="inlineStr">
-        <is>
-          <t>9981</t>
-        </is>
-      </c>
-      <c r="G17" s="316" t="inlineStr">
-        <is>
-          <t>50-71-02</t>
-        </is>
-      </c>
-      <c r="H17" s="315"/>
-      <c r="I17" s="315"/>
-      <c r="J17" s="315"/>
-      <c r="K17" s="315"/>
-      <c r="L17" s="315" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M17" s="315"/>
-      <c r="N17" s="315" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" customHeight="true" ht="30.0">
-      <c r="A18" s="315" t="inlineStr">
-        <is>
-          <t>1005007517486374</t>
-        </is>
-      </c>
-      <c r="B18" s="315" t="inlineStr">
-        <is>
-          <t>스팸6호 4세트 스팸 명절 추석 선물세트</t>
-        </is>
-      </c>
-      <c r="C18" s="315" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D18" s="315" t="inlineStr">
-        <is>
-          <t>12000041099568766</t>
-        </is>
-      </c>
-      <c r="E18" s="316" t="inlineStr">
-        <is>
-          <t>154500.00</t>
-        </is>
-      </c>
-      <c r="F18" s="316" t="inlineStr">
-        <is>
-          <t>9816</t>
-        </is>
-      </c>
-      <c r="G18" s="316" t="inlineStr">
-        <is>
-          <t>45-05</t>
-        </is>
-      </c>
-      <c r="H18" s="315"/>
-      <c r="I18" s="315"/>
-      <c r="J18" s="315"/>
-      <c r="K18" s="315"/>
-      <c r="L18" s="315" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M18" s="315"/>
-      <c r="N18" s="315" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" customHeight="true" ht="30.0">
-      <c r="A19" s="315" t="inlineStr">
-        <is>
-          <t>1005007517580171</t>
-        </is>
-      </c>
-      <c r="B19" s="315" t="inlineStr">
-        <is>
-          <t>스팸6호 1세트 스팸 명절 추석 선물세트</t>
-        </is>
-      </c>
-      <c r="C19" s="315" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D19" s="315" t="inlineStr">
-        <is>
-          <t>12000041099919070</t>
-        </is>
-      </c>
-      <c r="E19" s="316" t="inlineStr">
-        <is>
-          <t>41200.00</t>
-        </is>
-      </c>
-      <c r="F19" s="316" t="inlineStr">
-        <is>
-          <t>9916</t>
-        </is>
-      </c>
-      <c r="G19" s="316" t="inlineStr">
-        <is>
-          <t>45-05</t>
-        </is>
-      </c>
-      <c r="H19" s="315"/>
-      <c r="I19" s="315"/>
-      <c r="J19" s="315"/>
-      <c r="K19" s="315"/>
-      <c r="L19" s="315" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="315"/>
-      <c r="N19" s="315" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="true"/>
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(햄축산통조림_hide!$I$7,0,0,6,1)</formula1>
+      <formula1>OFFSET(통조림기타_hide!$I$7,0,0,5,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(햄축산통조림_hide!$K$7,0,0,2,1)</formula1>
+      <formula1>OFFSET(통조림기타_hide!$K$7,0,0,2,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -23245,7 +23321,7 @@
       </c>
       <c r="F6" s="43" t="inlineStr">
         <is>
-          <t>9842</t>
+          <t>9841</t>
         </is>
       </c>
       <c r="G6" s="43" t="inlineStr">
@@ -23349,7 +23425,7 @@
       </c>
       <c r="F8" s="43" t="inlineStr">
         <is>
-          <t>9767</t>
+          <t>9766</t>
         </is>
       </c>
       <c r="G8" s="43" t="inlineStr">
@@ -23609,7 +23685,7 @@
       </c>
       <c r="F13" s="43" t="inlineStr">
         <is>
-          <t>9929</t>
+          <t>9928</t>
         </is>
       </c>
       <c r="G13" s="43" t="inlineStr">
@@ -23869,7 +23945,7 @@
       </c>
       <c r="F18" s="43" t="inlineStr">
         <is>
-          <t>9941</t>
+          <t>9939</t>
         </is>
       </c>
       <c r="G18" s="43" t="inlineStr">
@@ -23921,7 +23997,7 @@
       </c>
       <c r="F19" s="43" t="inlineStr">
         <is>
-          <t>9951</t>
+          <t>9949</t>
         </is>
       </c>
       <c r="G19" s="43" t="inlineStr">
@@ -23973,7 +24049,7 @@
       </c>
       <c r="F20" s="43" t="inlineStr">
         <is>
-          <t>9985</t>
+          <t>9984</t>
         </is>
       </c>
       <c r="G20" s="43" t="inlineStr">
@@ -24077,7 +24153,7 @@
       </c>
       <c r="F22" s="43" t="inlineStr">
         <is>
-          <t>9776</t>
+          <t>9770</t>
         </is>
       </c>
       <c r="G22" s="43" t="inlineStr">
@@ -24181,7 +24257,7 @@
       </c>
       <c r="F24" s="43" t="inlineStr">
         <is>
-          <t>9681</t>
+          <t>9677</t>
         </is>
       </c>
       <c r="G24" s="43" t="inlineStr">
@@ -24285,7 +24361,7 @@
       </c>
       <c r="F26" s="43" t="inlineStr">
         <is>
-          <t>9881</t>
+          <t>9866</t>
         </is>
       </c>
       <c r="G26" s="43" t="inlineStr">
@@ -24545,7 +24621,7 @@
       </c>
       <c r="F31" s="43" t="inlineStr">
         <is>
-          <t>9859</t>
+          <t>9858</t>
         </is>
       </c>
       <c r="G31" s="43" t="inlineStr">
@@ -24805,7 +24881,7 @@
       </c>
       <c r="F36" s="43" t="inlineStr">
         <is>
-          <t>9995</t>
+          <t>9994</t>
         </is>
       </c>
       <c r="G36" s="43" t="inlineStr">
@@ -25052,7 +25128,7 @@
       <c r="H6"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J6"/>
@@ -25076,7 +25152,7 @@
       <c r="H7"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>병</t>
+          <t>포장</t>
         </is>
       </c>
       <c r="J7"/>
@@ -25100,7 +25176,7 @@
       <c r="H8"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>포장</t>
+          <t>Piece（단품）</t>
         </is>
       </c>
       <c r="J8"/>
@@ -25124,7 +25200,7 @@
       <c r="H9"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Piece（단품）</t>
+          <t>프로모션/기획 묶음</t>
         </is>
       </c>
       <c r="J9"/>
@@ -25148,7 +25224,7 @@
       <c r="H10"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>프로모션/기획 묶음</t>
+          <t>박스</t>
         </is>
       </c>
       <c r="J10"/>
@@ -25172,7 +25248,7 @@
       <c r="H11"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>박스</t>
+          <t>세트</t>
         </is>
       </c>
       <c r="J11"/>
@@ -25196,7 +25272,7 @@
       <c r="H12"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>세트</t>
+          <t>####splitter line####</t>
         </is>
       </c>
       <c r="J12"/>
@@ -25216,7 +25292,7 @@
       <c r="H13"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>####splitter line####</t>
+          <t>6512378</t>
         </is>
       </c>
       <c r="J13"/>
@@ -25236,7 +25312,7 @@
       <c r="H14"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3525584</t>
+          <t>7826584</t>
         </is>
       </c>
       <c r="J14"/>
@@ -25256,7 +25332,7 @@
       <c r="H15"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>6512378</t>
+          <t>12301206</t>
         </is>
       </c>
       <c r="J15"/>
@@ -25276,7 +25352,7 @@
       <c r="H16"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>7826584</t>
+          <t>23399605318</t>
         </is>
       </c>
       <c r="J16"/>
@@ -25296,7 +25372,7 @@
       <c r="H17"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>12301206</t>
+          <t>24087192969</t>
         </is>
       </c>
       <c r="J17"/>
@@ -25304,46 +25380,6 @@
       <c r="L17"/>
       <c r="M17"/>
       <c r="N17"/>
-    </row>
-    <row r="18">
-      <c r="A18"/>
-      <c r="B18"/>
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18"/>
-      <c r="F18"/>
-      <c r="G18"/>
-      <c r="H18"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>23399605318</t>
-        </is>
-      </c>
-      <c r="J18"/>
-      <c r="K18"/>
-      <c r="L18"/>
-      <c r="M18"/>
-      <c r="N18"/>
-    </row>
-    <row r="19">
-      <c r="A19"/>
-      <c r="B19"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>24087192969</t>
-        </is>
-      </c>
-      <c r="J19"/>
-      <c r="K19"/>
-      <c r="L19"/>
-      <c r="M19"/>
-      <c r="N19"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -25741,12 +25777,12 @@
     <row r="6" customHeight="true" ht="30.0">
       <c r="A6" s="336" t="inlineStr">
         <is>
-          <t>1005009937710715</t>
+          <t>1005007044473531</t>
         </is>
       </c>
       <c r="B6" s="336" t="inlineStr">
         <is>
-          <t>스팸 특별한선택 H-2호 5세트 선물세트</t>
+          <t>팔도 비빔면 멀티팩(5개입) 8개</t>
         </is>
       </c>
       <c r="C6" s="336" t="inlineStr">
@@ -25756,22 +25792,22 @@
       </c>
       <c r="D6" s="336" t="inlineStr">
         <is>
-          <t>12000050627105859</t>
+          <t>12000039205412355</t>
         </is>
       </c>
       <c r="E6" s="337" t="inlineStr">
         <is>
-          <t>79900.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="F6" s="337" t="inlineStr">
         <is>
-          <t>9996</t>
+          <t>9994</t>
         </is>
       </c>
       <c r="G6" s="337" t="inlineStr">
         <is>
-          <t>45-12-06</t>
+          <t>54-21</t>
         </is>
       </c>
       <c r="H6" s="336"/>
@@ -25793,12 +25829,12 @@
     <row r="7" customHeight="true" ht="30.0">
       <c r="A7" s="336" t="inlineStr">
         <is>
-          <t>1005009943428343</t>
+          <t>1005007044527555</t>
         </is>
       </c>
       <c r="B7" s="336" t="inlineStr">
         <is>
-          <t>스팸 특별한선택 H-2호 1세트 선물세트</t>
+          <t>오뚜기 진라면 매운맛 멀티팩(5개입) 8개</t>
         </is>
       </c>
       <c r="C7" s="336" t="inlineStr">
@@ -25808,22 +25844,22 @@
       </c>
       <c r="D7" s="336" t="inlineStr">
         <is>
-          <t>12000050643623167</t>
+          <t>12000039205101603</t>
         </is>
       </c>
       <c r="E7" s="337" t="inlineStr">
         <is>
-          <t>18700.00</t>
+          <t>28100.00</t>
         </is>
       </c>
       <c r="F7" s="337" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>9200</t>
         </is>
       </c>
       <c r="G7" s="337" t="inlineStr">
         <is>
-          <t>45-12-06</t>
+          <t>39-91</t>
         </is>
       </c>
       <c r="H7" s="336"/>
@@ -25845,12 +25881,12 @@
     <row r="8" customHeight="true" ht="30.0">
       <c r="A8" s="336" t="inlineStr">
         <is>
-          <t>1005009943395385</t>
+          <t>1005007044214904</t>
         </is>
       </c>
       <c r="B8" s="336" t="inlineStr">
         <is>
-          <t>스팸 12K호 1세트</t>
+          <t>팔도 왕뚜껑 컵라면 110g 18개</t>
         </is>
       </c>
       <c r="C8" s="336" t="inlineStr">
@@ -25860,22 +25896,22 @@
       </c>
       <c r="D8" s="336" t="inlineStr">
         <is>
-          <t>12000050643682021</t>
+          <t>12000039205264392</t>
         </is>
       </c>
       <c r="E8" s="337" t="inlineStr">
         <is>
-          <t>26500.00</t>
+          <t>23800.00</t>
         </is>
       </c>
       <c r="F8" s="337" t="inlineStr">
         <is>
-          <t>9997</t>
+          <t>9966</t>
         </is>
       </c>
       <c r="G8" s="337" t="inlineStr">
         <is>
-          <t>45-10-09</t>
+          <t>22-22</t>
         </is>
       </c>
       <c r="H8" s="336"/>
@@ -25897,12 +25933,12 @@
     <row r="9" customHeight="true" ht="30.0">
       <c r="A9" s="336" t="inlineStr">
         <is>
-          <t>1005009937638801</t>
+          <t>1005007044375655</t>
         </is>
       </c>
       <c r="B9" s="336" t="inlineStr">
         <is>
-          <t>스팸 12K호 4세트</t>
+          <t>팔도 김치왕뚜껑 컵라면 18입</t>
         </is>
       </c>
       <c r="C9" s="336" t="inlineStr">
@@ -25912,22 +25948,22 @@
       </c>
       <c r="D9" s="336" t="inlineStr">
         <is>
-          <t>12000050627038470</t>
+          <t>12000039205121918</t>
         </is>
       </c>
       <c r="E9" s="337" t="inlineStr">
         <is>
-          <t>95500.00</t>
+          <t>23900.00</t>
         </is>
       </c>
       <c r="F9" s="337" t="inlineStr">
         <is>
-          <t>9942</t>
+          <t>9994</t>
         </is>
       </c>
       <c r="G9" s="337" t="inlineStr">
         <is>
-          <t>45-10-09</t>
+          <t>22-23-01</t>
         </is>
       </c>
       <c r="H9" s="336"/>
@@ -25949,12 +25985,12 @@
     <row r="10" customHeight="true" ht="30.0">
       <c r="A10" s="336" t="inlineStr">
         <is>
-          <t>1005009937881801</t>
+          <t>1005007044267807</t>
         </is>
       </c>
       <c r="B10" s="336" t="inlineStr">
         <is>
-          <t>CJ 풍성한S호 3세트 선물세트</t>
+          <t>팔도 비빔면 컵라면 16입</t>
         </is>
       </c>
       <c r="C10" s="336" t="inlineStr">
@@ -25964,22 +26000,22 @@
       </c>
       <c r="D10" s="336" t="inlineStr">
         <is>
-          <t>12000050627580842</t>
+          <t>12000039205464212</t>
         </is>
       </c>
       <c r="E10" s="337" t="inlineStr">
         <is>
-          <t>133300.00</t>
+          <t>21500.00</t>
         </is>
       </c>
       <c r="F10" s="337" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>9972</t>
         </is>
       </c>
       <c r="G10" s="337" t="inlineStr">
         <is>
-          <t>45-09-01</t>
+          <t>54-21-03</t>
         </is>
       </c>
       <c r="H10" s="336"/>
@@ -25998,275 +26034,15 @@
         </is>
       </c>
     </row>
-    <row r="11" customHeight="true" ht="30.0">
-      <c r="A11" s="336" t="inlineStr">
-        <is>
-          <t>1005009943444204</t>
-        </is>
-      </c>
-      <c r="B11" s="336" t="inlineStr">
-        <is>
-          <t>청정원 스페셜 NH2호 1세트 선물세트</t>
-        </is>
-      </c>
-      <c r="C11" s="336" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D11" s="336" t="inlineStr">
-        <is>
-          <t>12000050643525722</t>
-        </is>
-      </c>
-      <c r="E11" s="337" t="inlineStr">
-        <is>
-          <t>27500.00</t>
-        </is>
-      </c>
-      <c r="F11" s="337" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G11" s="337" t="inlineStr">
-        <is>
-          <t>01-17</t>
-        </is>
-      </c>
-      <c r="H11" s="336"/>
-      <c r="I11" s="336"/>
-      <c r="J11" s="336"/>
-      <c r="K11" s="336"/>
-      <c r="L11" s="336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="336"/>
-      <c r="N11" s="336" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" customHeight="true" ht="30.0">
-      <c r="A12" s="336" t="inlineStr">
-        <is>
-          <t>1005009937891554</t>
-        </is>
-      </c>
-      <c r="B12" s="336" t="inlineStr">
-        <is>
-          <t>청정원 스페셜 NH2호 3세트 선물세트</t>
-        </is>
-      </c>
-      <c r="C12" s="336" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D12" s="336" t="inlineStr">
-        <is>
-          <t>12000050627562432</t>
-        </is>
-      </c>
-      <c r="E12" s="337" t="inlineStr">
-        <is>
-          <t>75700.00</t>
-        </is>
-      </c>
-      <c r="F12" s="337" t="inlineStr">
-        <is>
-          <t>9995</t>
-        </is>
-      </c>
-      <c r="G12" s="337" t="inlineStr">
-        <is>
-          <t>01-17</t>
-        </is>
-      </c>
-      <c r="H12" s="336"/>
-      <c r="I12" s="336"/>
-      <c r="J12" s="336"/>
-      <c r="K12" s="336"/>
-      <c r="L12" s="336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M12" s="336"/>
-      <c r="N12" s="336" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" customHeight="true" ht="30.0">
-      <c r="A13" s="336" t="inlineStr">
-        <is>
-          <t>1005009943250846</t>
-        </is>
-      </c>
-      <c r="B13" s="336" t="inlineStr">
-        <is>
-          <t>청정원 L6호 1세트 선물세트</t>
-        </is>
-      </c>
-      <c r="C13" s="336" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D13" s="336" t="inlineStr">
-        <is>
-          <t>12000050643481691</t>
-        </is>
-      </c>
-      <c r="E13" s="337" t="inlineStr">
-        <is>
-          <t>23200.00</t>
-        </is>
-      </c>
-      <c r="F13" s="337" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G13" s="337" t="inlineStr">
-        <is>
-          <t>01-19-06</t>
-        </is>
-      </c>
-      <c r="H13" s="336"/>
-      <c r="I13" s="336"/>
-      <c r="J13" s="336"/>
-      <c r="K13" s="336"/>
-      <c r="L13" s="336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M13" s="336"/>
-      <c r="N13" s="336" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" customHeight="true" ht="30.0">
-      <c r="A14" s="336" t="inlineStr">
-        <is>
-          <t>1005009937925088</t>
-        </is>
-      </c>
-      <c r="B14" s="336" t="inlineStr">
-        <is>
-          <t>청정원 L6호 4세트 선물세트</t>
-        </is>
-      </c>
-      <c r="C14" s="336" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D14" s="336" t="inlineStr">
-        <is>
-          <t>12000050627510269</t>
-        </is>
-      </c>
-      <c r="E14" s="337" t="inlineStr">
-        <is>
-          <t>82700.00</t>
-        </is>
-      </c>
-      <c r="F14" s="337" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G14" s="337" t="inlineStr">
-        <is>
-          <t>01-19-06</t>
-        </is>
-      </c>
-      <c r="H14" s="336"/>
-      <c r="I14" s="336"/>
-      <c r="J14" s="336"/>
-      <c r="K14" s="336"/>
-      <c r="L14" s="336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="336"/>
-      <c r="N14" s="336" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" customHeight="true" ht="30.0">
-      <c r="A15" s="336" t="inlineStr">
-        <is>
-          <t>1005007850275922</t>
-        </is>
-      </c>
-      <c r="B15" s="336" t="inlineStr">
-        <is>
-          <t>동표 을지로골뱅이 400g 24개</t>
-        </is>
-      </c>
-      <c r="C15" s="336" t="inlineStr">
-        <is>
-          <t>KRW</t>
-        </is>
-      </c>
-      <c r="D15" s="336" t="inlineStr">
-        <is>
-          <t>12000042534092495</t>
-        </is>
-      </c>
-      <c r="E15" s="337" t="inlineStr">
-        <is>
-          <t>189300.00</t>
-        </is>
-      </c>
-      <c r="F15" s="337" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="G15" s="337" t="inlineStr">
-        <is>
-          <t>46-04</t>
-        </is>
-      </c>
-      <c r="H15" s="336"/>
-      <c r="I15" s="336"/>
-      <c r="J15" s="336"/>
-      <c r="K15" s="336"/>
-      <c r="L15" s="336" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M15" s="336"/>
-      <c r="N15" s="336" t="inlineStr">
-        <is>
-          <t>absolute</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <sheetCalcPr fullCalcOnLoad="true"/>
   <sheetProtection insertColumns="true" deleteColumns="false" formatCells="false" formatColumns="false" formatRows="true" autoFilter="false" deleteRows="false" insertRows="false" insertHyperlinks="false" objects="true" selectLockedCells="false" selectUnlockedCells="false" scenarios="true" sort="false" password="9D43" sheet="true"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="I5:I32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(통조림기타_hide!$I$7,0,0,5,1)</formula1>
+      <formula1>OFFSET(컵라면_hide!$I$7,0,0,5,1)</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="K5:K32768" allowBlank="true" errorStyle="stop" showErrorMessage="true" showInputMessage="true">
-      <formula1>OFFSET(통조림기타_hide!$K$7,0,0,2,1)</formula1>
+      <formula1>OFFSET(컵라면_hide!$K$7,0,0,2,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -30462,7 +30238,7 @@
       </c>
       <c r="F7" s="421" t="inlineStr">
         <is>
-          <t>9945</t>
+          <t>9943</t>
         </is>
       </c>
       <c r="G7" s="421" t="inlineStr">
@@ -32065,7 +31841,7 @@
       </c>
       <c r="F8" s="442" t="inlineStr">
         <is>
-          <t>9986</t>
+          <t>9985</t>
         </is>
       </c>
       <c r="G8" s="442" t="inlineStr">
@@ -36876,7 +36652,7 @@
       </c>
       <c r="F8" s="64" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>886</t>
         </is>
       </c>
       <c r="G8" s="64" t="inlineStr">
@@ -37100,7 +36876,7 @@
       </c>
       <c r="F12" s="64" t="inlineStr">
         <is>
-          <t>9946</t>
+          <t>9945</t>
         </is>
       </c>
       <c r="G12" s="64" t="inlineStr">
@@ -37360,7 +37136,7 @@
       </c>
       <c r="F17" s="64" t="inlineStr">
         <is>
-          <t>8858</t>
+          <t>8857</t>
         </is>
       </c>
       <c r="G17" s="64" t="inlineStr">
@@ -38088,7 +37864,7 @@
       </c>
       <c r="F31" s="64" t="inlineStr">
         <is>
-          <t>9750</t>
+          <t>9747</t>
         </is>
       </c>
       <c r="G31" s="64" t="inlineStr">
@@ -38660,7 +38436,7 @@
       </c>
       <c r="F42" s="64" t="inlineStr">
         <is>
-          <t>9964</t>
+          <t>9962</t>
         </is>
       </c>
       <c r="G42" s="64" t="inlineStr">
@@ -39180,7 +38956,7 @@
       </c>
       <c r="F52" s="64" t="inlineStr">
         <is>
-          <t>9439</t>
+          <t>9436</t>
         </is>
       </c>
       <c r="G52" s="64" t="inlineStr">

</xml_diff>